<commit_message>
updates on analysis engine
</commit_message>
<xml_diff>
--- a/P012-excavator-split_data_files/06_07_2017_Yared_excavator_records_part_1.xlsx
+++ b/P012-excavator-split_data_files/06_07_2017_Yared_excavator_records_part_1.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="excavator" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="mpdm" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="daily_variables" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="excavator" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="mpdm" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="daily_variables" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1197,7 +1197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z106"/>
+  <dimension ref="A1:Z111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.875" customWidth="1" min="1" max="1"/>
@@ -7373,6 +7373,221 @@
       <c r="X106" s="10" t="n"/>
       <c r="Y106" s="10" t="n"/>
       <c r="Z106" s="10" t="n"/>
+    </row>
+    <row r="107">
+      <c r="E107" t="n">
+        <v>5</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>1/14 foreman:1 opetator ,1 helper</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Hoe</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">soft rock excavation using hydraulic excavator </t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>soft rock</t>
+        </is>
+      </c>
+      <c r="K107" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="L107" t="n">
+        <v>45</v>
+      </c>
+      <c r="M107" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="N107" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="Q107" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="R107" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="E108" t="n">
+        <v>5</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>1/14 foreman:1 opetator ,1 helper</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Hoe</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">soft rock excavation using hydraulic excavator </t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>soft rock</t>
+        </is>
+      </c>
+      <c r="K108" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="L108" t="n">
+        <v>45</v>
+      </c>
+      <c r="M108" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="N108" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="Q108" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="R108" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="E109" t="n">
+        <v>5</v>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>1/14 foreman:1 opetator ,1 helper</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Hoe</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">soft rock excavation using hydraulic excavator </t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>soft rock</t>
+        </is>
+      </c>
+      <c r="K109" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="L109" t="n">
+        <v>45</v>
+      </c>
+      <c r="M109" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="N109" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="Q109" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="R109" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="E110" t="n">
+        <v>5</v>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>1/14 foreman:1 opetator ,1 helper</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Hoe</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">soft rock excavation using hydraulic excavator </t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>soft rock</t>
+        </is>
+      </c>
+      <c r="K110" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="L110" t="n">
+        <v>45</v>
+      </c>
+      <c r="M110" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="N110" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="Q110" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="R110" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="E111" t="n">
+        <v>5</v>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>1/14 foreman:1 opetator ,1 helper</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Hoe</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">soft rock excavation using hydraulic excavator </t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>soft rock</t>
+        </is>
+      </c>
+      <c r="K111" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="L111" t="n">
+        <v>45</v>
+      </c>
+      <c r="M111" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="N111" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="Q111" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="R111" t="n">
+        <v>21</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -12390,7 +12605,7 @@
       </c>
       <c r="H21" s="69" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="I21" s="67" t="n"/>

</xml_diff>

<commit_message>
separating ui from engine
</commit_message>
<xml_diff>
--- a/P012-excavator-split_data_files/06_07_2017_Yared_excavator_records_part_1.xlsx
+++ b/P012-excavator-split_data_files/06_07_2017_Yared_excavator_records_part_1.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="excavator" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="mpdm" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="daily_variables" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="excavator" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="mpdm" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="daily_variables" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1197,7 +1197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z111"/>
+  <dimension ref="A1:Z106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.875" customWidth="1" min="1" max="1"/>
@@ -7373,221 +7373,6 @@
       <c r="X106" s="10" t="n"/>
       <c r="Y106" s="10" t="n"/>
       <c r="Z106" s="10" t="n"/>
-    </row>
-    <row r="107">
-      <c r="E107" t="n">
-        <v>5</v>
-      </c>
-      <c r="F107" t="inlineStr">
-        <is>
-          <t>1/14 foreman:1 opetator ,1 helper</t>
-        </is>
-      </c>
-      <c r="G107" t="inlineStr">
-        <is>
-          <t>Hoe</t>
-        </is>
-      </c>
-      <c r="H107" t="inlineStr">
-        <is>
-          <t xml:space="preserve">soft rock excavation using hydraulic excavator </t>
-        </is>
-      </c>
-      <c r="J107" t="inlineStr">
-        <is>
-          <t>soft rock</t>
-        </is>
-      </c>
-      <c r="K107" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="L107" t="n">
-        <v>45</v>
-      </c>
-      <c r="M107" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="N107" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="Q107" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="R107" t="n">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="108">
-      <c r="E108" t="n">
-        <v>5</v>
-      </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>1/14 foreman:1 opetator ,1 helper</t>
-        </is>
-      </c>
-      <c r="G108" t="inlineStr">
-        <is>
-          <t>Hoe</t>
-        </is>
-      </c>
-      <c r="H108" t="inlineStr">
-        <is>
-          <t xml:space="preserve">soft rock excavation using hydraulic excavator </t>
-        </is>
-      </c>
-      <c r="J108" t="inlineStr">
-        <is>
-          <t>soft rock</t>
-        </is>
-      </c>
-      <c r="K108" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="L108" t="n">
-        <v>45</v>
-      </c>
-      <c r="M108" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="N108" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="Q108" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="R108" t="n">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="109">
-      <c r="E109" t="n">
-        <v>5</v>
-      </c>
-      <c r="F109" t="inlineStr">
-        <is>
-          <t>1/14 foreman:1 opetator ,1 helper</t>
-        </is>
-      </c>
-      <c r="G109" t="inlineStr">
-        <is>
-          <t>Hoe</t>
-        </is>
-      </c>
-      <c r="H109" t="inlineStr">
-        <is>
-          <t xml:space="preserve">soft rock excavation using hydraulic excavator </t>
-        </is>
-      </c>
-      <c r="J109" t="inlineStr">
-        <is>
-          <t>soft rock</t>
-        </is>
-      </c>
-      <c r="K109" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="L109" t="n">
-        <v>45</v>
-      </c>
-      <c r="M109" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="N109" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="Q109" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="R109" t="n">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="110">
-      <c r="E110" t="n">
-        <v>5</v>
-      </c>
-      <c r="F110" t="inlineStr">
-        <is>
-          <t>1/14 foreman:1 opetator ,1 helper</t>
-        </is>
-      </c>
-      <c r="G110" t="inlineStr">
-        <is>
-          <t>Hoe</t>
-        </is>
-      </c>
-      <c r="H110" t="inlineStr">
-        <is>
-          <t xml:space="preserve">soft rock excavation using hydraulic excavator </t>
-        </is>
-      </c>
-      <c r="J110" t="inlineStr">
-        <is>
-          <t>soft rock</t>
-        </is>
-      </c>
-      <c r="K110" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="L110" t="n">
-        <v>45</v>
-      </c>
-      <c r="M110" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="N110" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="Q110" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="R110" t="n">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="111">
-      <c r="E111" t="n">
-        <v>5</v>
-      </c>
-      <c r="F111" t="inlineStr">
-        <is>
-          <t>1/14 foreman:1 opetator ,1 helper</t>
-        </is>
-      </c>
-      <c r="G111" t="inlineStr">
-        <is>
-          <t>Hoe</t>
-        </is>
-      </c>
-      <c r="H111" t="inlineStr">
-        <is>
-          <t xml:space="preserve">soft rock excavation using hydraulic excavator </t>
-        </is>
-      </c>
-      <c r="J111" t="inlineStr">
-        <is>
-          <t>soft rock</t>
-        </is>
-      </c>
-      <c r="K111" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="L111" t="n">
-        <v>45</v>
-      </c>
-      <c r="M111" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="N111" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="Q111" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="R111" t="n">
-        <v>21</v>
-      </c>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -12605,7 +12390,7 @@
       </c>
       <c r="H21" s="69" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="I21" s="67" t="n"/>

</xml_diff>